<commit_message>
feat: subrasante + corte/escarpe + canal + pasarela + adoquin + rotonda + zapata muro
Nuevas categorias viales (5):
  corte      → excavacion_en_corte (m³ = area × prof_media)
  escarpe    → escarpe_y_limpieza (m² directa)
  canal      → canal_hormigon_revestido (ml = area / ancho)
  pasarela   → hormigon + acero + moldaje (tablero liviano e=25cm)
  adoquin    → pavimento_adoquin_hormigon (m² directa)
  rotonda    → alias calzada (agrega ROTONDA|GLORIETA al regex)

Mejoras a formulas existentes:
  calzada    → subrasante_estabilizada m² cuando subrasante_m > 0 (default 0.15m)
               excavacion incluye subrasante en paquete total
  muro       → zapata hormigon cuando zapata_factor > 0 (default 0.0)

Resultado Ruta 1: 19 partidas, $20,134 MM CLP (+0.7% vs referencial MOP $20,000 MM)
Tests: 107/107 (12 nuevos)
Precios CSV: +6 nuevas partidas (total 45)

https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/ruta1_cubicacion.xlsx
+++ b/ruta1_cubicacion.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-18 02:22</t>
+          <t>2026-05-18 02:29</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$ 12.410.232.000</t>
+          <t>$ 13.535.412.000</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$ 3.102.558.000</t>
+          <t>$ 3.383.853.000</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$ 15.512.790.000</t>
+          <t>$ 16.919.265.000</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$ 2.947.430.100</t>
+          <t>$ 3.214.660.350</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>$ 18.460.220.100 CLP</t>
+          <t>$ 20.133.925.350 CLP</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$ 43.305 CLP/m²</t>
+          <t>$ 47.231 CLP/m²</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1325,24 +1325,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>excavacion_tierra_comun</t>
+          <t>subrasante_estabilizada</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Excavacion tierra comun</t>
+          <t>Subrasante estabilizada e=150mm</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>90804</v>
+        <v>197400</v>
       </c>
       <c r="E7" t="n">
-        <v>8000</v>
+        <v>4500</v>
       </c>
       <c r="F7">
         <f>D7*E7</f>
@@ -1357,24 +1357,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cuneta_hormigon_revestida</t>
+          <t>excavacion_tierra_comun</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cuneta hormigon revestida a=0.60m</t>
+          <t>Excavacion tierra comun</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>42000</v>
+        <v>120414</v>
       </c>
       <c r="E8" t="n">
-        <v>45000</v>
+        <v>8000</v>
       </c>
       <c r="F8">
         <f>D8*E8</f>
@@ -1389,24 +1389,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>excavacion_tunel_roca</t>
+          <t>cuneta_hormigon_revestida</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Excavacion tunel 9.0×6.0 m</t>
+          <t>Cuneta hormigon revestida a=0.60m</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9720</v>
+        <v>42000</v>
       </c>
       <c r="E9" t="n">
-        <v>85000</v>
+        <v>45000</v>
       </c>
       <c r="F9">
         <f>D9*E9</f>
@@ -1421,24 +1421,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>revestimiento_tunel_hormigon</t>
+          <t>excavacion_tunel_roca</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Revestimiento tunel hormigon e=45cm</t>
+          <t>Excavacion tunel 9.0×6.0 m</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5400</v>
+        <v>9720</v>
       </c>
       <c r="E10" t="n">
-        <v>120000</v>
+        <v>85000</v>
       </c>
       <c r="F10">
         <f>D10*E10</f>
@@ -1453,24 +1453,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>acero_refuerzo_a630</t>
+          <t>revestimiento_tunel_hormigon</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Acero refuerzo A630-42H</t>
+          <t>Revestimiento tunel hormigon e=45cm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>388800</v>
+        <v>5400</v>
       </c>
       <c r="E11" t="n">
-        <v>1200</v>
+        <v>120000</v>
       </c>
       <c r="F11">
         <f>D11*E11</f>
@@ -1485,24 +1485,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>muro_contencion_hormigon</t>
+          <t>acero_refuerzo_a630</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Muro de contencion hormigon e=45cm</t>
+          <t>Acero refuerzo A630-42H</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4500</v>
+        <v>388800</v>
       </c>
       <c r="E12" t="n">
-        <v>95000</v>
+        <v>1200</v>
       </c>
       <c r="F12">
         <f>D12*E12</f>
@@ -1517,24 +1517,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hormigon_armado_H30</t>
+          <t>muro_contencion_hormigon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hormigon armado H30 muro e=45cm</t>
+          <t>Muro de contencion hormigon e=45cm</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2025</v>
+        <v>4500</v>
       </c>
       <c r="E13" t="n">
-        <v>380000</v>
+        <v>95000</v>
       </c>
       <c r="F13">
         <f>D13*E13</f>
@@ -1549,24 +1549,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>moldaje_muro</t>
+          <t>hormigon_armado_H30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Moldaje muro</t>
+          <t>Hormigon armado H30 muro e=45cm</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9000</v>
+        <v>2025</v>
       </c>
       <c r="E14" t="n">
-        <v>25000</v>
+        <v>380000</v>
       </c>
       <c r="F14">
         <f>D14*E14</f>
@@ -1581,12 +1581,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>demarcacion_vial_termoplastico</t>
+          <t>moldaje_muro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Demarcacion vial termoplastico</t>
+          <t>Moldaje muro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1595,10 +1595,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50400</v>
+        <v>9000</v>
       </c>
       <c r="E15" t="n">
-        <v>8000</v>
+        <v>25000</v>
       </c>
       <c r="F15">
         <f>D15*E15</f>
@@ -1613,24 +1613,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>senal_vial_retrorreflectante</t>
+          <t>demarcacion_vial_termoplastico</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Senal vial retroreflectante (1.5m²/señal)</t>
+          <t>Demarcacion vial termoplastico</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>560</v>
+        <v>50400</v>
       </c>
       <c r="E16" t="n">
-        <v>180000</v>
+        <v>8000</v>
       </c>
       <c r="F16">
         <f>D16*E16</f>
@@ -1645,12 +1645,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>luminaria_led_vial</t>
+          <t>senal_vial_retrorreflectante</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Luminaria LED vial (poste + luminaria + instalacion)</t>
+          <t>Senal vial retroreflectante (1.5m²/señal)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1659,10 +1659,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1050</v>
+        <v>560</v>
       </c>
       <c r="E17" t="n">
-        <v>480000</v>
+        <v>180000</v>
       </c>
       <c r="F17">
         <f>D17*E17</f>
@@ -1677,24 +1677,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>guardavia_flexible_w</t>
+          <t>luminaria_led_vial</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Guardavia flexible W-beam doble ola</t>
+          <t>Luminaria LED vial (poste + luminaria + instalacion)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8400</v>
+        <v>1050</v>
       </c>
       <c r="E18" t="n">
-        <v>32000</v>
+        <v>480000</v>
       </c>
       <c r="F18">
         <f>D18*E18</f>
@@ -1709,24 +1709,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>terraplen_compactado</t>
+          <t>guardavia_flexible_w</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Terraplen compactado h_media=1.8m</t>
+          <t>Guardavia flexible W-beam doble ola</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>175770</v>
+        <v>8400</v>
       </c>
       <c r="E19" t="n">
-        <v>6000</v>
+        <v>32000</v>
       </c>
       <c r="F19">
         <f>D19*E19</f>
@@ -1741,24 +1741,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>alcantarilla_marco_hormigon</t>
+          <t>terraplen_compactado</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alcantarilla marco hormigon a=1.5m</t>
+          <t>Terraplen compactado h_media=1.8m</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1008</v>
+        <v>175770</v>
       </c>
       <c r="E20" t="n">
-        <v>450000</v>
+        <v>6000</v>
       </c>
       <c r="F20">
         <f>D20*E20</f>
@@ -1773,24 +1773,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>revegetacion_hidrosiembra</t>
+          <t>alcantarilla_marco_hormigon</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Revegetacion hidrosiembra taludes</t>
+          <t>Alcantarilla marco hormigon a=1.5m</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>37800</v>
+        <v>1008</v>
       </c>
       <c r="E21" t="n">
-        <v>3500</v>
+        <v>450000</v>
       </c>
       <c r="F21">
         <f>D21*E21</f>
@@ -1802,58 +1802,90 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>revegetacion_hidrosiembra</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revegetacion hidrosiembra taludes</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>37800</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F22">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ONDAC 2026Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>SUBTOTAL NETO</t>
         </is>
       </c>
-      <c r="F23" s="3">
-        <f>SUM(F2:F21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" t="inlineStr">
+      <c r="F24" s="3">
+        <f>SUM(F2:F22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
         <is>
           <t>GG + Utilidad (25%)</t>
         </is>
       </c>
-      <c r="F24">
-        <f>F23*0.25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+      <c r="F25">
+        <f>F24*0.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>SUBTOTAL + GG&amp;U</t>
         </is>
       </c>
-      <c r="F25" s="3">
-        <f>F23+F24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
+      <c r="F26" s="3">
+        <f>F24+F25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
         <is>
           <t>IVA (19%)</t>
         </is>
       </c>
-      <c r="F26">
-        <f>F25*0.19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="8" t="inlineStr">
+      <c r="F27">
+        <f>F26*0.19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>TOTAL CON IVA</t>
         </is>
       </c>
-      <c r="F27" s="4">
-        <f>F25+F26</f>
+      <c r="F28" s="4">
+        <f>F26+F27</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: colector PVC/hormigon + berma → calzada + paso superior/bajo nivel
- Nueva categoria 'colector': colector_pvc_300mm o colector_hormigon_600mm
  segun keyword; ml = area / ancho_zanja_m (default 0.80m)
- BERMA incluida en regex calzada (era keyword muerto en _VIALES)
- PASO SUPERIOR VEHICULAR y PASO BAJO NIVEL → categoria puente
- _VIALES regex expandido: COLECTOR, TUBERIA, ALCANTARILLADO, DREN, PASO SUPERIOR
- secciones_civiles.yaml: nueva seccion 'colector'
- demo_ruta1.py: agrega COLECTOR PVC DRENAJE LONGITUDINAL (8,400 ml)
- Total estimacion Ruta 1: $21.2 MM CLP (+6% vs $20,000 MM referencial)
- 5 tests nuevos (total 119/119)

https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/ruta1_cubicacion.xlsx
+++ b/ruta1_cubicacion.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-18 02:38</t>
+          <t>2026-05-18 02:44</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>426282.0 m²</t>
+          <t>433002.0 m²</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>426282.0 m²</t>
+          <t>433002.0 m²</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$ 13.535.412.000</t>
+          <t>$ 14.249.412.000</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$ 3.383.853.000</t>
+          <t>$ 3.562.353.000</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$ 16.919.265.000</t>
+          <t>$ 17.811.765.000</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$ 3.214.660.350</t>
+          <t>$ 3.384.235.350</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>$ 20.133.925.350 CLP</t>
+          <t>$ 21.196.000.350 CLP</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$ 47.231 CLP/m²</t>
+          <t>$ 48.951 CLP/m²</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -780,7 +780,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CUNETA REVESTIDA HORMIGON</t>
+          <t>COLECTOR PVC DRENAJE LONGITUDINAL</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -789,13 +789,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25200</v>
+        <v>6720</v>
       </c>
       <c r="E4" t="n">
-        <v>648.0700000000001</v>
+        <v>334.66</v>
       </c>
       <c r="F4" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DEMARCACION VIAL CALZADA</t>
+          <t>CUNETA REVESTIDA HORMIGON</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -820,13 +820,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>50400</v>
+        <v>25200</v>
       </c>
       <c r="E5" t="n">
-        <v>916.52</v>
+        <v>648.0700000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GUARDAVIA FLEXIBLE W KM0-KM21</t>
+          <t>DEMARCACION VIAL CALZADA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -851,13 +851,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4200</v>
+        <v>50400</v>
       </c>
       <c r="E6" t="n">
-        <v>264.58</v>
+        <v>916.52</v>
       </c>
       <c r="F6" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ILUMINACION VIAL RUTA 1</t>
+          <t>GUARDAVIA FLEXIBLE W KM0-KM21</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MIRADOR CALZADA KM210</t>
+          <t>ILUMINACION VIAL RUTA 1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -913,13 +913,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>480</v>
+        <v>4200</v>
       </c>
       <c r="E8" t="n">
-        <v>89.44</v>
+        <v>264.58</v>
       </c>
       <c r="F8" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MIRADOR CALZADA KM213</t>
+          <t>MIRADOR CALZADA KM210</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MURO DE CONTENCION HORMIGON</t>
+          <t>MIRADOR CALZADA KM213</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -975,13 +975,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4500</v>
+        <v>480</v>
       </c>
       <c r="E10" t="n">
-        <v>273.86</v>
+        <v>89.44</v>
       </c>
       <c r="F10" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -997,7 +997,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REVEGETACION TALUDES</t>
+          <t>MURO DE CONTENCION HORMIGON</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37800</v>
+        <v>4500</v>
       </c>
       <c r="E11" t="n">
-        <v>793.73</v>
+        <v>273.86</v>
       </c>
       <c r="F11" t="n">
-        <v>0.78</v>
+        <v>0.85</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SENALETIVA VERTICAL KM0-KM21</t>
+          <t>REVEGETACION TALUDES</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1037,13 +1037,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>840</v>
+        <v>37800</v>
       </c>
       <c r="E12" t="n">
-        <v>118.32</v>
+        <v>793.73</v>
       </c>
       <c r="F12" t="n">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SOBREANCHO CURVAS PISTA</t>
+          <t>SENALETIVA VERTICAL KM0-KM21</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1068,13 +1068,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2100</v>
+        <v>840</v>
       </c>
       <c r="E13" t="n">
-        <v>187.08</v>
+        <v>118.32</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TERRAPLEN COMPACTADO</t>
+          <t>SOBREANCHO CURVAS PISTA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1099,10 +1099,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>97650</v>
+        <v>2100</v>
       </c>
       <c r="E14" t="n">
-        <v>1275.74</v>
+        <v>187.08</v>
       </c>
       <c r="F14" t="n">
         <v>0.8</v>
@@ -1121,37 +1121,68 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>TERRAPLEN COMPACTADO</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>vial</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>97650</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1275.74</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ruta 1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>TUNEL GALLEGUILLOS</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>vial</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>1620</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E16" t="n">
         <v>378</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F16" t="n">
         <v>0.9</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Subtotal Ruta 1</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
-        <v>426282</v>
+      <c r="D17" s="3" t="n">
+        <v>433002</v>
       </c>
     </row>
   </sheetData>
@@ -1165,7 +1196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1834,58 +1865,90 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>colector_pvc_300mm</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Colector PVC 300mm (0.80m zanja)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E23" t="n">
+        <v>85000</v>
+      </c>
+      <c r="F23">
+        <f>D23*E23</f>
+        <v/>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ONDAC 2026Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>SUBTOTAL NETO</t>
         </is>
       </c>
-      <c r="F24" s="3">
-        <f>SUM(F2:F22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" t="inlineStr">
+      <c r="F25" s="3">
+        <f>SUM(F2:F23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
         <is>
           <t>GG + Utilidad (25%)</t>
         </is>
       </c>
-      <c r="F25">
-        <f>F24*0.25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
+      <c r="F26">
+        <f>F25*0.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>SUBTOTAL + GG&amp;U</t>
         </is>
       </c>
-      <c r="F26" s="3">
-        <f>F24+F25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="inlineStr">
+      <c r="F27" s="3">
+        <f>F25+F26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
         <is>
           <t>IVA (19%)</t>
         </is>
       </c>
-      <c r="F27">
-        <f>F26*0.19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="8" t="inlineStr">
+      <c r="F28">
+        <f>F27*0.19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>TOTAL CON IVA</t>
         </is>
       </c>
-      <c r="F28" s="4">
-        <f>F26+F27</f>
+      <c r="F29" s="4">
+        <f>F27+F28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: eliminar doble conteo en muro — ahora usa precio all-inclusive m2
Antes: muro_contencion_hormigon m2 + hormigon_armado m3 + acero kg + moldaje m2
  → $335,400/m² cara (3.5× el precio de mercado)

Ahora: solo muro_contencion_hormigon m2 (precio ONDAC all-inclusive $95,000/m²)
  → Consistente con cuneta, vereda, adoquin, ciclovia

Impacto demo Ruta 1: $21.2 MM → $19.4 MM CLP (-3% vs $20,000 MM referencial MOP)
- Geotextil trasdos sigue como partida adicional opcional (no incluida en m2)
- Tests actualizados (131/131)

https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/ruta1_cubicacion.xlsx
+++ b/ruta1_cubicacion.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-18 02:44</t>
+          <t>2026-05-18 02:57</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$ 14.249.412.000</t>
+          <t>$ 13.036.212.000</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$ 3.562.353.000</t>
+          <t>$ 3.259.053.000</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$ 17.811.765.000</t>
+          <t>$ 16.295.265.000</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$ 3.384.235.350</t>
+          <t>$ 3.096.100.350</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>$ 21.196.000.350 CLP</t>
+          <t>$ 19.391.365.350 CLP</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$ 48.951 CLP/m²</t>
+          <t>$ 44.783 CLP/m²</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>388800</v>
+        <v>206550</v>
       </c>
       <c r="E12" t="n">
         <v>1200</v>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Muro de contencion hormigon e=45cm</t>
+          <t>Muro de contencion hormigon (all-inclusive)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1580,24 +1580,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hormigon_armado_H30</t>
+          <t>demarcacion_vial_termoplastico</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hormigon armado H30 muro e=45cm</t>
+          <t>Demarcacion vial termoplastico</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2025</v>
+        <v>50400</v>
       </c>
       <c r="E14" t="n">
-        <v>380000</v>
+        <v>8000</v>
       </c>
       <c r="F14">
         <f>D14*E14</f>
@@ -1612,24 +1612,24 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>moldaje_muro</t>
+          <t>senal_vial_retrorreflectante</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Moldaje muro</t>
+          <t>Senal vial retroreflectante (1.5m²/señal)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9000</v>
+        <v>560</v>
       </c>
       <c r="E15" t="n">
-        <v>25000</v>
+        <v>180000</v>
       </c>
       <c r="F15">
         <f>D15*E15</f>
@@ -1644,24 +1644,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>demarcacion_vial_termoplastico</t>
+          <t>luminaria_led_vial</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Demarcacion vial termoplastico</t>
+          <t>Luminaria LED vial (poste + luminaria + instalacion)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50400</v>
+        <v>1050</v>
       </c>
       <c r="E16" t="n">
-        <v>8000</v>
+        <v>480000</v>
       </c>
       <c r="F16">
         <f>D16*E16</f>
@@ -1676,24 +1676,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>senal_vial_retrorreflectante</t>
+          <t>guardavia_flexible_w</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Senal vial retroreflectante (1.5m²/señal)</t>
+          <t>Guardavia flexible W-beam doble ola</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>560</v>
+        <v>8400</v>
       </c>
       <c r="E17" t="n">
-        <v>180000</v>
+        <v>32000</v>
       </c>
       <c r="F17">
         <f>D17*E17</f>
@@ -1708,24 +1708,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>luminaria_led_vial</t>
+          <t>terraplen_compactado</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Luminaria LED vial (poste + luminaria + instalacion)</t>
+          <t>Terraplen compactado h_media=1.8m</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1050</v>
+        <v>175770</v>
       </c>
       <c r="E18" t="n">
-        <v>480000</v>
+        <v>6000</v>
       </c>
       <c r="F18">
         <f>D18*E18</f>
@@ -1740,12 +1740,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>guardavia_flexible_w</t>
+          <t>alcantarilla_marco_hormigon</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Guardavia flexible W-beam doble ola</t>
+          <t>Alcantarilla marco hormigon a=1.5m</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1754,10 +1754,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8400</v>
+        <v>1008</v>
       </c>
       <c r="E19" t="n">
-        <v>32000</v>
+        <v>450000</v>
       </c>
       <c r="F19">
         <f>D19*E19</f>
@@ -1772,24 +1772,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>terraplen_compactado</t>
+          <t>revegetacion_hidrosiembra</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Terraplen compactado h_media=1.8m</t>
+          <t>Revegetacion hidrosiembra taludes</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>175770</v>
+        <v>37800</v>
       </c>
       <c r="E20" t="n">
-        <v>6000</v>
+        <v>3500</v>
       </c>
       <c r="F20">
         <f>D20*E20</f>
@@ -1804,12 +1804,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>alcantarilla_marco_hormigon</t>
+          <t>colector_pvc_300mm</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alcantarilla marco hormigon a=1.5m</t>
+          <t>Colector PVC 300mm (0.80m zanja)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1818,10 +1818,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1008</v>
+        <v>8400</v>
       </c>
       <c r="E21" t="n">
-        <v>450000</v>
+        <v>85000</v>
       </c>
       <c r="F21">
         <f>D21*E21</f>
@@ -1833,122 +1833,58 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>revegetacion_hidrosiembra</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revegetacion hidrosiembra taludes</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>37800</v>
-      </c>
-      <c r="E22" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F22">
-        <f>D22*E22</f>
-        <v/>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>ONDAC 2026Q1</t>
-        </is>
-      </c>
-    </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>colector_pvc_300mm</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Colector PVC 300mm (0.80m zanja)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>8400</v>
-      </c>
-      <c r="E23" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F23">
-        <f>D23*E23</f>
-        <v/>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>ONDAC 2026Q1</t>
-        </is>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>SUBTOTAL NETO</t>
+        </is>
+      </c>
+      <c r="F23" s="3">
+        <f>SUM(F2:F21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GG + Utilidad (25%)</t>
+        </is>
+      </c>
+      <c r="F24">
+        <f>F23*0.25</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>SUBTOTAL NETO</t>
+          <t>SUBTOTAL + GG&amp;U</t>
         </is>
       </c>
       <c r="F25" s="3">
-        <f>SUM(F2:F23)</f>
+        <f>F23+F24</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>GG + Utilidad (25%)</t>
+          <t>IVA (19%)</t>
         </is>
       </c>
       <c r="F26">
-        <f>F25*0.25</f>
+        <f>F25*0.19</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>SUBTOTAL + GG&amp;U</t>
-        </is>
-      </c>
-      <c r="F27" s="3">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL CON IVA</t>
+        </is>
+      </c>
+      <c r="F27" s="4">
         <f>F25+F26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>IVA (19%)</t>
-        </is>
-      </c>
-      <c r="F28">
-        <f>F27*0.19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL CON IVA</t>
-        </is>
-      </c>
-      <c r="F29" s="4">
-        <f>F27+F28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerar excel ruta1 demo
https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/ruta1_cubicacion.xlsx
+++ b/ruta1_cubicacion.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-18 03:37</t>
+          <t>2026-05-18 03:48</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1976,37 +1976,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>RECINTOS CON CLASIFICACION HEURISTICA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Categoria asignada</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>GUARDAVIA FLEXIBLE W KM0-KM21</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>vial</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>